<commit_message>
update: data PNL x0.75
</commit_message>
<xml_diff>
--- a/data/PNL.xlsx
+++ b/data/PNL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\financial_automation\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E82B3E72-566B-4192-AB7E-DBB5D771E83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97F20557-7446-4F27-83ED-BC7DEF80F067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="345" windowWidth="11340" windowHeight="15600" xr2:uid="{FC1DE28B-20D4-4352-B81C-69B33F180141}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{FC1DE28B-20D4-4352-B81C-69B33F180141}"/>
   </bookViews>
   <sheets>
     <sheet name="Profit and Loss" sheetId="2" r:id="rId1"/>
@@ -1985,43 +1985,43 @@
       <c r="F9" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="G9" s="16">
+      <c r="G9" s="5">
         <v>888459419</v>
       </c>
-      <c r="H9" s="16">
+      <c r="H9" s="5">
         <v>1217170381</v>
       </c>
-      <c r="I9" s="16">
+      <c r="I9" s="5">
         <v>825738230</v>
       </c>
-      <c r="J9" s="16">
+      <c r="J9" s="5">
         <v>847205372</v>
       </c>
-      <c r="K9" s="16">
+      <c r="K9" s="5">
         <v>658628003</v>
       </c>
-      <c r="L9" s="16">
+      <c r="L9" s="5">
         <v>1560885538</v>
       </c>
-      <c r="M9" s="16">
+      <c r="M9" s="5">
         <v>1160125848</v>
       </c>
-      <c r="N9" s="16">
+      <c r="N9" s="5">
         <v>2624558250</v>
       </c>
-      <c r="O9" s="16">
+      <c r="O9" s="5">
         <v>1681875116</v>
       </c>
-      <c r="P9" s="16">
+      <c r="P9" s="5">
         <v>890790424</v>
       </c>
-      <c r="Q9" s="16">
+      <c r="Q9" s="5">
         <v>780543323</v>
       </c>
-      <c r="R9" s="16">
+      <c r="R9" s="5">
         <v>598525337</v>
       </c>
-      <c r="S9" s="16">
+      <c r="S9" s="5">
         <v>395585406</v>
       </c>
     </row>
@@ -2109,43 +2109,43 @@
       <c r="F12" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G12" s="16">
+      <c r="G12" s="5">
         <v>392859588</v>
       </c>
-      <c r="H12" s="16">
+      <c r="H12" s="5">
         <v>567297057</v>
       </c>
-      <c r="I12" s="16">
+      <c r="I12" s="5">
         <v>318033700</v>
       </c>
-      <c r="J12" s="16">
+      <c r="J12" s="5">
         <v>703769948</v>
       </c>
-      <c r="K12" s="16">
+      <c r="K12" s="5">
         <v>836427700</v>
       </c>
-      <c r="L12" s="16">
+      <c r="L12" s="5">
         <v>1076625000</v>
       </c>
-      <c r="M12" s="16">
+      <c r="M12" s="5">
         <v>1164660528</v>
       </c>
-      <c r="N12" s="16">
+      <c r="N12" s="5">
         <v>1436936043</v>
       </c>
-      <c r="O12" s="16">
+      <c r="O12" s="5">
         <v>997836775</v>
       </c>
-      <c r="P12" s="16">
+      <c r="P12" s="5">
         <v>678869108</v>
       </c>
-      <c r="Q12" s="16">
+      <c r="Q12" s="5">
         <v>773775186</v>
       </c>
-      <c r="R12" s="16">
+      <c r="R12" s="5">
         <v>634740499</v>
       </c>
-      <c r="S12" s="16">
+      <c r="S12" s="5">
         <v>331996489</v>
       </c>
     </row>
@@ -2153,43 +2153,43 @@
       <c r="F13" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="G13" s="16">
-        <v>0</v>
-      </c>
-      <c r="H13" s="16">
+      <c r="G13" s="5">
+        <v>0</v>
+      </c>
+      <c r="H13" s="5">
         <v>116850000</v>
       </c>
-      <c r="I13" s="16">
+      <c r="I13" s="5">
         <v>24490000</v>
       </c>
-      <c r="J13" s="16">
+      <c r="J13" s="5">
         <v>41192000</v>
       </c>
-      <c r="K13" s="16">
+      <c r="K13" s="5">
         <v>81813694</v>
       </c>
-      <c r="L13" s="16">
+      <c r="L13" s="5">
         <v>330117286</v>
       </c>
-      <c r="M13" s="16">
+      <c r="M13" s="5">
         <v>111534500</v>
       </c>
-      <c r="N13" s="16">
+      <c r="N13" s="5">
         <v>87260000</v>
       </c>
-      <c r="O13" s="16">
+      <c r="O13" s="5">
         <v>105817780</v>
       </c>
-      <c r="P13" s="16">
+      <c r="P13" s="5">
         <v>87130000</v>
       </c>
-      <c r="Q13" s="16">
+      <c r="Q13" s="5">
         <v>49087500</v>
       </c>
-      <c r="R13" s="16">
+      <c r="R13" s="5">
         <v>47700000</v>
       </c>
-      <c r="S13" s="16">
+      <c r="S13" s="5">
         <v>33990000</v>
       </c>
     </row>
@@ -2277,43 +2277,43 @@
       <c r="F16" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="G16" s="16">
+      <c r="G16" s="5">
         <v>104743600</v>
       </c>
-      <c r="H16" s="16">
+      <c r="H16" s="5">
         <v>163176759</v>
       </c>
-      <c r="I16" s="16">
+      <c r="I16" s="5">
         <v>95422100</v>
       </c>
-      <c r="J16" s="16">
+      <c r="J16" s="5">
         <v>104327240</v>
       </c>
-      <c r="K16" s="16">
+      <c r="K16" s="5">
         <v>153894020</v>
       </c>
-      <c r="L16" s="16">
+      <c r="L16" s="5">
         <v>230057258</v>
       </c>
-      <c r="M16" s="16">
+      <c r="M16" s="5">
         <v>231799416</v>
       </c>
-      <c r="N16" s="16">
+      <c r="N16" s="5">
         <v>261099557</v>
       </c>
-      <c r="O16" s="16">
+      <c r="O16" s="5">
         <v>233044290</v>
       </c>
-      <c r="P16" s="16">
+      <c r="P16" s="5">
         <v>113041928</v>
       </c>
-      <c r="Q16" s="16">
+      <c r="Q16" s="5">
         <v>144337500</v>
       </c>
-      <c r="R16" s="16">
+      <c r="R16" s="5">
         <v>151771820</v>
       </c>
-      <c r="S16" s="16">
+      <c r="S16" s="5">
         <v>85356500</v>
       </c>
     </row>
@@ -2321,43 +2321,43 @@
       <c r="F17" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="G17" s="16">
-        <v>0</v>
-      </c>
-      <c r="H17" s="16">
-        <v>0</v>
-      </c>
-      <c r="I17" s="16">
-        <v>0</v>
-      </c>
-      <c r="J17" s="16">
-        <v>0</v>
-      </c>
-      <c r="K17" s="16">
+      <c r="G17" s="5">
+        <v>0</v>
+      </c>
+      <c r="H17" s="5">
+        <v>0</v>
+      </c>
+      <c r="I17" s="5">
+        <v>0</v>
+      </c>
+      <c r="J17" s="5">
+        <v>0</v>
+      </c>
+      <c r="K17" s="5">
         <v>3256195</v>
       </c>
-      <c r="L17" s="16">
+      <c r="L17" s="5">
         <v>122400526</v>
       </c>
-      <c r="M17" s="16">
+      <c r="M17" s="5">
         <v>1500000</v>
       </c>
-      <c r="N17" s="16">
-        <v>0</v>
-      </c>
-      <c r="O17" s="16">
+      <c r="N17" s="5">
+        <v>0</v>
+      </c>
+      <c r="O17" s="5">
         <v>9289253</v>
       </c>
-      <c r="P17" s="16">
+      <c r="P17" s="5">
         <v>55080000</v>
       </c>
-      <c r="Q17" s="16">
-        <v>0</v>
-      </c>
-      <c r="R17" s="16">
-        <v>0</v>
-      </c>
-      <c r="S17" s="16">
+      <c r="Q17" s="5">
+        <v>0</v>
+      </c>
+      <c r="R17" s="5">
+        <v>0</v>
+      </c>
+      <c r="S17" s="5">
         <v>0</v>
       </c>
     </row>
@@ -2445,43 +2445,43 @@
       <c r="F20" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="G20" s="16">
+      <c r="G20" s="5">
         <v>30374300</v>
       </c>
-      <c r="H20" s="16">
+      <c r="H20" s="5">
         <v>110172669</v>
       </c>
-      <c r="I20" s="16">
+      <c r="I20" s="5">
         <v>22831445</v>
       </c>
-      <c r="J20" s="16">
+      <c r="J20" s="5">
         <v>71502401</v>
       </c>
-      <c r="K20" s="16">
+      <c r="K20" s="5">
         <v>82195144</v>
       </c>
-      <c r="L20" s="16">
+      <c r="L20" s="5">
         <v>159228714</v>
       </c>
-      <c r="M20" s="16">
+      <c r="M20" s="5">
         <v>145170250</v>
       </c>
-      <c r="N20" s="16">
+      <c r="N20" s="5">
         <v>176283600</v>
       </c>
-      <c r="O20" s="16">
+      <c r="O20" s="5">
         <v>233803909</v>
       </c>
-      <c r="P20" s="16">
+      <c r="P20" s="5">
         <v>104085500</v>
       </c>
-      <c r="Q20" s="16">
+      <c r="Q20" s="5">
         <v>99619481</v>
       </c>
-      <c r="R20" s="16">
+      <c r="R20" s="5">
         <v>96309872</v>
       </c>
-      <c r="S20" s="16">
+      <c r="S20" s="5">
         <v>58030820</v>
       </c>
     </row>
@@ -2569,43 +2569,43 @@
       <c r="F23" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="G23" s="16">
+      <c r="G23" s="5">
         <v>6555000</v>
       </c>
-      <c r="H23" s="16">
+      <c r="H23" s="5">
         <v>9918000</v>
       </c>
-      <c r="I23" s="16">
+      <c r="I23" s="5">
         <v>7105000</v>
       </c>
-      <c r="J23" s="16">
+      <c r="J23" s="5">
         <v>7984200</v>
       </c>
-      <c r="K23" s="16">
+      <c r="K23" s="5">
         <v>6664000</v>
       </c>
-      <c r="L23" s="16">
+      <c r="L23" s="5">
         <v>17710900</v>
       </c>
-      <c r="M23" s="16">
+      <c r="M23" s="5">
         <v>16454400</v>
       </c>
-      <c r="N23" s="16">
+      <c r="N23" s="5">
         <v>21600000</v>
       </c>
-      <c r="O23" s="16">
+      <c r="O23" s="5">
         <v>23500800</v>
       </c>
-      <c r="P23" s="16">
+      <c r="P23" s="5">
         <v>10712200</v>
       </c>
-      <c r="Q23" s="16">
+      <c r="Q23" s="5">
         <v>12434000</v>
       </c>
-      <c r="R23" s="16">
+      <c r="R23" s="5">
         <v>4491700</v>
       </c>
-      <c r="S23" s="16">
+      <c r="S23" s="5">
         <v>4907600</v>
       </c>
     </row>
@@ -2693,43 +2693,43 @@
       <c r="F26" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="G26" s="16">
+      <c r="G26" s="5">
         <v>40411000</v>
       </c>
-      <c r="H26" s="16">
+      <c r="H26" s="5">
         <v>57246000</v>
       </c>
-      <c r="I26" s="16">
+      <c r="I26" s="5">
         <v>53116500</v>
       </c>
-      <c r="J26" s="16">
+      <c r="J26" s="5">
         <v>56483814</v>
       </c>
-      <c r="K26" s="16">
+      <c r="K26" s="5">
         <v>80627498</v>
       </c>
-      <c r="L26" s="16">
+      <c r="L26" s="5">
         <v>100992800</v>
       </c>
-      <c r="M26" s="16">
+      <c r="M26" s="5">
         <v>129272520</v>
       </c>
-      <c r="N26" s="16">
+      <c r="N26" s="5">
         <v>139573000</v>
       </c>
-      <c r="O26" s="16">
+      <c r="O26" s="5">
         <v>147731399</v>
       </c>
-      <c r="P26" s="16">
+      <c r="P26" s="5">
         <v>56470000</v>
       </c>
-      <c r="Q26" s="16">
+      <c r="Q26" s="5">
         <v>42855000</v>
       </c>
-      <c r="R26" s="16">
+      <c r="R26" s="5">
         <v>53339222</v>
       </c>
-      <c r="S26" s="16">
+      <c r="S26" s="5">
         <v>39241500</v>
       </c>
     </row>
@@ -2817,43 +2817,43 @@
       <c r="F29" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="G29" s="16">
+      <c r="G29" s="5">
         <v>4228182</v>
       </c>
-      <c r="H29" s="16">
+      <c r="H29" s="5">
         <v>750000</v>
       </c>
-      <c r="I29" s="16">
+      <c r="I29" s="5">
         <v>2822775</v>
       </c>
-      <c r="J29" s="16">
+      <c r="J29" s="5">
         <v>460995</v>
       </c>
-      <c r="K29" s="16">
+      <c r="K29" s="5">
         <v>9815861</v>
       </c>
-      <c r="L29" s="16">
+      <c r="L29" s="5">
         <v>22687237</v>
       </c>
-      <c r="M29" s="16">
+      <c r="M29" s="5">
         <v>5117400</v>
       </c>
-      <c r="N29" s="16">
+      <c r="N29" s="5">
         <v>34001497</v>
       </c>
-      <c r="O29" s="16">
+      <c r="O29" s="5">
         <v>23555790</v>
       </c>
-      <c r="P29" s="16">
+      <c r="P29" s="5">
         <v>6675200</v>
       </c>
-      <c r="Q29" s="16">
+      <c r="Q29" s="5">
         <v>7150000</v>
       </c>
-      <c r="R29" s="16">
+      <c r="R29" s="5">
         <v>6163164</v>
       </c>
-      <c r="S29" s="16">
+      <c r="S29" s="5">
         <v>8314820</v>
       </c>
     </row>
@@ -2861,43 +2861,43 @@
       <c r="F30" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="G30" s="16">
+      <c r="G30" s="5">
         <v>750000</v>
       </c>
-      <c r="H30" s="16">
-        <v>0</v>
-      </c>
-      <c r="I30" s="16">
+      <c r="H30" s="5">
+        <v>0</v>
+      </c>
+      <c r="I30" s="5">
         <v>900000</v>
       </c>
-      <c r="J30" s="16">
+      <c r="J30" s="5">
         <v>2150000</v>
       </c>
-      <c r="K30" s="16">
+      <c r="K30" s="5">
         <v>247934</v>
       </c>
-      <c r="L30" s="16">
+      <c r="L30" s="5">
         <v>3500000</v>
       </c>
-      <c r="M30" s="16">
+      <c r="M30" s="5">
         <v>123967</v>
       </c>
-      <c r="N30" s="16">
+      <c r="N30" s="5">
         <v>2800000</v>
       </c>
-      <c r="O30" s="16">
+      <c r="O30" s="5">
         <v>6450412</v>
       </c>
-      <c r="P30" s="16">
+      <c r="P30" s="5">
         <v>827000</v>
       </c>
-      <c r="Q30" s="16">
+      <c r="Q30" s="5">
         <v>398000</v>
       </c>
-      <c r="R30" s="16">
+      <c r="R30" s="5">
         <v>21479250</v>
       </c>
-      <c r="S30" s="16">
+      <c r="S30" s="5">
         <v>14602000</v>
       </c>
     </row>
@@ -2905,43 +2905,43 @@
       <c r="F31" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G31" s="16">
+      <c r="G31" s="5">
         <v>77000</v>
       </c>
-      <c r="H31" s="16">
+      <c r="H31" s="5">
         <v>757872</v>
       </c>
-      <c r="I31" s="16">
+      <c r="I31" s="5">
         <v>230720</v>
       </c>
-      <c r="J31" s="16">
+      <c r="J31" s="5">
         <v>1671610</v>
       </c>
-      <c r="K31" s="16">
+      <c r="K31" s="5">
         <v>5769920</v>
       </c>
-      <c r="L31" s="16">
+      <c r="L31" s="5">
         <v>1131200</v>
       </c>
-      <c r="M31" s="16">
+      <c r="M31" s="5">
         <v>1338400</v>
       </c>
-      <c r="N31" s="16">
+      <c r="N31" s="5">
         <v>3114530</v>
       </c>
-      <c r="O31" s="16">
+      <c r="O31" s="5">
         <v>2570600</v>
       </c>
-      <c r="P31" s="16">
+      <c r="P31" s="5">
         <v>1965600</v>
       </c>
-      <c r="Q31" s="16">
+      <c r="Q31" s="5">
         <v>1495200</v>
       </c>
-      <c r="R31" s="16">
+      <c r="R31" s="5">
         <v>393120</v>
       </c>
-      <c r="S31" s="16">
+      <c r="S31" s="5">
         <v>0</v>
       </c>
     </row>
@@ -2949,43 +2949,43 @@
       <c r="F32" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="G32" s="16">
+      <c r="G32" s="5">
         <v>865374073.39999998</v>
       </c>
-      <c r="H32" s="16">
+      <c r="H32" s="5">
         <v>865374073.39999998</v>
       </c>
-      <c r="I32" s="16">
+      <c r="I32" s="5">
         <v>865374073.39999998</v>
       </c>
-      <c r="J32" s="16">
+      <c r="J32" s="5">
         <v>761566667</v>
       </c>
-      <c r="K32" s="16">
+      <c r="K32" s="5">
         <v>761566667</v>
       </c>
-      <c r="L32" s="16">
+      <c r="L32" s="5">
         <v>761566667</v>
       </c>
-      <c r="M32" s="16">
+      <c r="M32" s="5">
         <v>761566667</v>
       </c>
-      <c r="N32" s="16">
+      <c r="N32" s="5">
         <v>761566667</v>
       </c>
-      <c r="O32" s="16">
+      <c r="O32" s="5">
         <v>761566667</v>
       </c>
-      <c r="P32" s="16">
+      <c r="P32" s="5">
         <v>761566667</v>
       </c>
-      <c r="Q32" s="16">
+      <c r="Q32" s="5">
         <v>761566667</v>
       </c>
-      <c r="R32" s="16">
+      <c r="R32" s="5">
         <v>761566667</v>
       </c>
-      <c r="S32" s="16">
+      <c r="S32" s="5">
         <v>761566667</v>
       </c>
     </row>
@@ -2993,43 +2993,43 @@
       <c r="F33" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="G33" s="16">
-        <v>0</v>
-      </c>
-      <c r="H33" s="16">
-        <v>0</v>
-      </c>
-      <c r="I33" s="16">
-        <v>0</v>
-      </c>
-      <c r="J33" s="16">
+      <c r="G33" s="5">
+        <v>0</v>
+      </c>
+      <c r="H33" s="5">
+        <v>0</v>
+      </c>
+      <c r="I33" s="5">
+        <v>0</v>
+      </c>
+      <c r="J33" s="5">
         <v>264762604</v>
       </c>
-      <c r="K33" s="16">
+      <c r="K33" s="5">
         <v>264762604</v>
       </c>
-      <c r="L33" s="16">
+      <c r="L33" s="5">
         <v>264762604</v>
       </c>
-      <c r="M33" s="16">
+      <c r="M33" s="5">
         <v>264762604</v>
       </c>
-      <c r="N33" s="16">
+      <c r="N33" s="5">
         <v>264762604</v>
       </c>
-      <c r="O33" s="16">
+      <c r="O33" s="5">
         <v>264762604</v>
       </c>
-      <c r="P33" s="16">
+      <c r="P33" s="5">
         <v>264762604</v>
       </c>
-      <c r="Q33" s="16">
+      <c r="Q33" s="5">
         <v>264762604</v>
       </c>
-      <c r="R33" s="16">
+      <c r="R33" s="5">
         <v>264762604</v>
       </c>
-      <c r="S33" s="16">
+      <c r="S33" s="5">
         <v>264762604</v>
       </c>
     </row>
@@ -3212,43 +3212,43 @@
       <c r="F39" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="G39" s="16">
+      <c r="G39" s="5">
         <v>149090086.28999999</v>
       </c>
-      <c r="H39" s="16">
+      <c r="H39" s="5">
         <v>235997948.16</v>
       </c>
-      <c r="I39" s="16">
+      <c r="I39" s="5">
         <v>158543265.59999999</v>
       </c>
-      <c r="J39" s="16">
+      <c r="J39" s="5">
         <v>242075531.28999999</v>
       </c>
-      <c r="K39" s="16">
+      <c r="K39" s="5">
         <v>302232573</v>
       </c>
-      <c r="L39" s="16">
+      <c r="L39" s="5">
         <v>396139623.44</v>
       </c>
-      <c r="M39" s="16">
+      <c r="M39" s="5">
         <v>367478998.36000001</v>
       </c>
-      <c r="N39" s="16">
+      <c r="N39" s="5">
         <v>475902251.94</v>
       </c>
-      <c r="O39" s="16">
+      <c r="O39" s="5">
         <v>367747663.94</v>
       </c>
-      <c r="P39" s="16">
+      <c r="P39" s="5">
         <v>226815505.81999999</v>
       </c>
-      <c r="Q39" s="16">
+      <c r="Q39" s="5">
         <v>288264643.70999998</v>
       </c>
-      <c r="R39" s="16">
+      <c r="R39" s="5">
         <v>198507374.69999999</v>
       </c>
-      <c r="S39" s="16">
+      <c r="S39" s="5">
         <v>94495562.700000003</v>
       </c>
     </row>
@@ -3256,43 +3256,43 @@
       <c r="F40" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="G40" s="16">
-        <v>0</v>
-      </c>
-      <c r="H40" s="16">
+      <c r="G40" s="5">
+        <v>0</v>
+      </c>
+      <c r="H40" s="5">
         <v>42350000</v>
       </c>
-      <c r="I40" s="16">
-        <v>0</v>
-      </c>
-      <c r="J40" s="16">
-        <v>0</v>
-      </c>
-      <c r="K40" s="16">
-        <v>0</v>
-      </c>
-      <c r="L40" s="16">
-        <v>8104150</v>
-      </c>
-      <c r="M40" s="16">
+      <c r="I40" s="5">
+        <v>0</v>
+      </c>
+      <c r="J40" s="5">
+        <v>0</v>
+      </c>
+      <c r="K40" s="5">
+        <v>0</v>
+      </c>
+      <c r="L40" s="5">
+        <v>8104149.9999999991</v>
+      </c>
+      <c r="M40" s="5">
         <v>750000</v>
       </c>
-      <c r="N40" s="16">
-        <v>0</v>
-      </c>
-      <c r="O40" s="16">
+      <c r="N40" s="5">
+        <v>0</v>
+      </c>
+      <c r="O40" s="5">
         <v>707200</v>
       </c>
-      <c r="P40" s="16">
+      <c r="P40" s="5">
         <v>1900260</v>
       </c>
-      <c r="Q40" s="16">
+      <c r="Q40" s="5">
         <v>7580000</v>
       </c>
-      <c r="R40" s="16">
+      <c r="R40" s="5">
         <v>748200</v>
       </c>
-      <c r="S40" s="16">
+      <c r="S40" s="5">
         <v>0</v>
       </c>
     </row>
@@ -3380,43 +3380,43 @@
       <c r="F43" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="G43" s="16">
+      <c r="G43" s="5">
         <v>27176942.91</v>
       </c>
-      <c r="H43" s="16">
+      <c r="H43" s="5">
         <v>40265654.439999998</v>
       </c>
-      <c r="I43" s="16">
+      <c r="I43" s="5">
         <v>28637761.02</v>
       </c>
-      <c r="J43" s="16">
+      <c r="J43" s="5">
         <v>31863292.199999999</v>
       </c>
-      <c r="K43" s="16">
+      <c r="K43" s="5">
         <v>41151475.479999997</v>
       </c>
-      <c r="L43" s="16">
+      <c r="L43" s="5">
         <v>77888215.439999998</v>
       </c>
-      <c r="M43" s="16">
+      <c r="M43" s="5">
         <v>56489302.939999998</v>
       </c>
-      <c r="N43" s="16">
+      <c r="N43" s="5">
         <v>78941731.620000005</v>
       </c>
-      <c r="O43" s="16">
+      <c r="O43" s="5">
         <v>69861939.700000003</v>
       </c>
-      <c r="P43" s="16">
+      <c r="P43" s="5">
         <v>43374093</v>
       </c>
-      <c r="Q43" s="16">
+      <c r="Q43" s="5">
         <v>37856951.159999996</v>
       </c>
-      <c r="R43" s="16">
+      <c r="R43" s="5">
         <v>43005192.890000001</v>
       </c>
-      <c r="S43" s="16">
+      <c r="S43" s="5">
         <v>18300527.890000001</v>
       </c>
     </row>
@@ -3424,43 +3424,43 @@
       <c r="F44" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="G44" s="16">
-        <v>0</v>
-      </c>
-      <c r="H44" s="16">
-        <v>0</v>
-      </c>
-      <c r="I44" s="16">
-        <v>0</v>
-      </c>
-      <c r="J44" s="16">
-        <v>0</v>
-      </c>
-      <c r="K44" s="16">
-        <v>0</v>
-      </c>
-      <c r="L44" s="16">
-        <v>0</v>
-      </c>
-      <c r="M44" s="16">
-        <v>0</v>
-      </c>
-      <c r="N44" s="16">
-        <v>0</v>
-      </c>
-      <c r="O44" s="16">
+      <c r="G44" s="5">
+        <v>0</v>
+      </c>
+      <c r="H44" s="5">
+        <v>0</v>
+      </c>
+      <c r="I44" s="5">
+        <v>0</v>
+      </c>
+      <c r="J44" s="5">
+        <v>0</v>
+      </c>
+      <c r="K44" s="5">
+        <v>0</v>
+      </c>
+      <c r="L44" s="5">
+        <v>0</v>
+      </c>
+      <c r="M44" s="5">
+        <v>0</v>
+      </c>
+      <c r="N44" s="5">
+        <v>0</v>
+      </c>
+      <c r="O44" s="5">
         <v>4432000</v>
       </c>
-      <c r="P44" s="16">
-        <v>0</v>
-      </c>
-      <c r="Q44" s="16">
-        <v>0</v>
-      </c>
-      <c r="R44" s="16">
-        <v>0</v>
-      </c>
-      <c r="S44" s="16">
+      <c r="P44" s="5">
+        <v>0</v>
+      </c>
+      <c r="Q44" s="5">
+        <v>0</v>
+      </c>
+      <c r="R44" s="5">
+        <v>0</v>
+      </c>
+      <c r="S44" s="5">
         <v>0</v>
       </c>
     </row>
@@ -3571,44 +3571,44 @@
       <c r="F48" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="G48" s="16">
+      <c r="G48" s="5">
         <v>1193384.18</v>
       </c>
-      <c r="H48" s="16">
+      <c r="H48" s="5">
         <v>1639993.71</v>
       </c>
-      <c r="I48" s="16">
+      <c r="I48" s="5">
         <v>2278666.29</v>
       </c>
-      <c r="J48" s="16">
+      <c r="J48" s="5">
         <v>1856216</v>
       </c>
-      <c r="K48" s="16">
+      <c r="K48" s="5">
         <v>2007080.22</v>
       </c>
-      <c r="L48" s="16">
+      <c r="L48" s="5">
         <v>2055523.96</v>
       </c>
-      <c r="M48" s="16">
+      <c r="M48" s="5">
         <v>3036578.92</v>
       </c>
-      <c r="N48" s="16">
+      <c r="N48" s="5">
         <v>4862016.7</v>
       </c>
-      <c r="O48" s="16">
+      <c r="O48" s="5">
         <v>4989176.2</v>
       </c>
-      <c r="P48" s="16">
+      <c r="P48" s="5">
         <v>3766350.09</v>
       </c>
-      <c r="Q48" s="16">
+      <c r="Q48" s="5">
         <v>2430034.1800000002</v>
       </c>
-      <c r="R48" s="16">
+      <c r="R48" s="5">
         <v>2918332.72</v>
       </c>
-      <c r="S48" s="16">
-        <v>1934151.8</v>
+      <c r="S48" s="5">
+        <v>1934151.8000000003</v>
       </c>
     </row>
     <row r="49" spans="1:19" ht="10.9" customHeight="1" x14ac:dyDescent="0.2">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="S49" s="17">
         <f t="shared" si="10"/>
-        <v>1934151.8</v>
+        <v>1934151.8000000003</v>
       </c>
     </row>
     <row r="50" spans="1:19" ht="10.9" customHeight="1" x14ac:dyDescent="0.2">
@@ -3695,43 +3695,43 @@
       <c r="F51" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="G51" s="16">
+      <c r="G51" s="5">
         <v>1140000</v>
       </c>
-      <c r="H51" s="16">
+      <c r="H51" s="5">
         <v>1145000</v>
       </c>
-      <c r="I51" s="16">
+      <c r="I51" s="5">
         <v>1110000</v>
       </c>
-      <c r="J51" s="16">
+      <c r="J51" s="5">
         <v>2530000</v>
       </c>
-      <c r="K51" s="16">
+      <c r="K51" s="5">
         <v>2385000</v>
       </c>
-      <c r="L51" s="16">
+      <c r="L51" s="5">
         <v>3720000</v>
       </c>
-      <c r="M51" s="16">
+      <c r="M51" s="5">
         <v>4320000</v>
       </c>
-      <c r="N51" s="16">
+      <c r="N51" s="5">
         <v>3350000</v>
       </c>
-      <c r="O51" s="16">
+      <c r="O51" s="5">
         <v>12330240</v>
       </c>
-      <c r="P51" s="16">
+      <c r="P51" s="5">
         <v>10528660</v>
       </c>
-      <c r="Q51" s="16">
+      <c r="Q51" s="5">
         <v>3730200</v>
       </c>
-      <c r="R51" s="16">
+      <c r="R51" s="5">
         <v>1347510</v>
       </c>
-      <c r="S51" s="16">
+      <c r="S51" s="5">
         <v>1472280</v>
       </c>
     </row>
@@ -3819,43 +3819,43 @@
       <c r="F54" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="G54" s="16">
+      <c r="G54" s="5">
         <v>20970000</v>
       </c>
-      <c r="H54" s="16">
+      <c r="H54" s="5">
         <v>99125000</v>
       </c>
-      <c r="I54" s="16">
-        <v>16000000</v>
-      </c>
-      <c r="J54" s="16">
+      <c r="I54" s="5">
+        <v>15999999.999999998</v>
+      </c>
+      <c r="J54" s="5">
         <v>36093885</v>
       </c>
-      <c r="K54" s="16">
+      <c r="K54" s="5">
         <v>73506115</v>
       </c>
-      <c r="L54" s="16">
-        <v>125765000</v>
-      </c>
-      <c r="M54" s="16">
+      <c r="L54" s="5">
+        <v>125764999.99999999</v>
+      </c>
+      <c r="M54" s="5">
         <v>101740000</v>
       </c>
-      <c r="N54" s="16">
-        <v>126582500</v>
-      </c>
-      <c r="O54" s="16">
+      <c r="N54" s="5">
+        <v>126582499.99999999</v>
+      </c>
+      <c r="O54" s="5">
         <v>164270000</v>
       </c>
-      <c r="P54" s="16">
+      <c r="P54" s="5">
         <v>74095000</v>
       </c>
-      <c r="Q54" s="16">
+      <c r="Q54" s="5">
         <v>38070000</v>
       </c>
-      <c r="R54" s="16">
-        <v>66490000</v>
-      </c>
-      <c r="S54" s="16">
+      <c r="R54" s="5">
+        <v>66489999.999999993</v>
+      </c>
+      <c r="S54" s="5">
         <v>39525000</v>
       </c>
     </row>
@@ -3863,43 +3863,43 @@
       <c r="F55" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="G55" s="16">
-        <v>0</v>
-      </c>
-      <c r="H55" s="16">
-        <v>0</v>
-      </c>
-      <c r="I55" s="16">
-        <v>0</v>
-      </c>
-      <c r="J55" s="16">
-        <v>0</v>
-      </c>
-      <c r="K55" s="16">
-        <v>0</v>
-      </c>
-      <c r="L55" s="16">
+      <c r="G55" s="5">
+        <v>0</v>
+      </c>
+      <c r="H55" s="5">
+        <v>0</v>
+      </c>
+      <c r="I55" s="5">
+        <v>0</v>
+      </c>
+      <c r="J55" s="5">
+        <v>0</v>
+      </c>
+      <c r="K55" s="5">
+        <v>0</v>
+      </c>
+      <c r="L55" s="5">
         <v>3500000</v>
       </c>
-      <c r="M55" s="16">
-        <v>0</v>
-      </c>
-      <c r="N55" s="16">
-        <v>0</v>
-      </c>
-      <c r="O55" s="16">
+      <c r="M55" s="5">
+        <v>0</v>
+      </c>
+      <c r="N55" s="5">
+        <v>0</v>
+      </c>
+      <c r="O55" s="5">
         <v>3500000</v>
       </c>
-      <c r="P55" s="16">
+      <c r="P55" s="5">
         <v>200000</v>
       </c>
-      <c r="Q55" s="16">
+      <c r="Q55" s="5">
         <v>6150000</v>
       </c>
-      <c r="R55" s="16">
+      <c r="R55" s="5">
         <v>5000000</v>
       </c>
-      <c r="S55" s="16">
+      <c r="S55" s="5">
         <v>19425000</v>
       </c>
     </row>
@@ -3907,43 +3907,43 @@
       <c r="F56" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="G56" s="16">
-        <v>0</v>
-      </c>
-      <c r="H56" s="16">
-        <v>480000</v>
-      </c>
-      <c r="I56" s="16">
+      <c r="G56" s="5">
+        <v>0</v>
+      </c>
+      <c r="H56" s="5">
+        <v>479999.99999999994</v>
+      </c>
+      <c r="I56" s="5">
         <v>420000</v>
       </c>
-      <c r="J56" s="16">
-        <v>0</v>
-      </c>
-      <c r="K56" s="16">
+      <c r="J56" s="5">
+        <v>0</v>
+      </c>
+      <c r="K56" s="5">
         <v>6375000</v>
       </c>
-      <c r="L56" s="16">
-        <v>0</v>
-      </c>
-      <c r="M56" s="16">
-        <v>0</v>
-      </c>
-      <c r="N56" s="16">
-        <v>0</v>
-      </c>
-      <c r="O56" s="16">
+      <c r="L56" s="5">
+        <v>0</v>
+      </c>
+      <c r="M56" s="5">
+        <v>0</v>
+      </c>
+      <c r="N56" s="5">
+        <v>0</v>
+      </c>
+      <c r="O56" s="5">
         <v>600000</v>
       </c>
-      <c r="P56" s="16">
-        <v>0</v>
-      </c>
-      <c r="Q56" s="16">
+      <c r="P56" s="5">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="5">
         <v>360000</v>
       </c>
-      <c r="R56" s="16">
+      <c r="R56" s="5">
         <v>1200000</v>
       </c>
-      <c r="S56" s="16">
+      <c r="S56" s="5">
         <v>0</v>
       </c>
     </row>
@@ -3961,7 +3961,7 @@
       </c>
       <c r="I57" s="17">
         <f t="shared" si="12"/>
-        <v>16420000</v>
+        <v>16419999.999999998</v>
       </c>
       <c r="J57" s="17">
         <f t="shared" si="12"/>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="L57" s="17">
         <f t="shared" si="12"/>
-        <v>129265000</v>
+        <v>129264999.99999999</v>
       </c>
       <c r="M57" s="17">
         <f t="shared" si="12"/>
@@ -3981,7 +3981,7 @@
       </c>
       <c r="N57" s="17">
         <f t="shared" si="12"/>
-        <v>126582500</v>
+        <v>126582499.99999999</v>
       </c>
       <c r="O57" s="17">
         <f t="shared" si="12"/>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="L58" s="17">
         <f t="shared" si="13"/>
-        <v>135040523.96000001</v>
+        <v>135040523.95999998</v>
       </c>
       <c r="M58" s="17">
         <f t="shared" si="13"/>
@@ -4087,7 +4087,7 @@
       </c>
       <c r="L59" s="17">
         <f t="shared" si="14"/>
-        <v>617172512.84000003</v>
+        <v>617172512.83999991</v>
       </c>
       <c r="M59" s="17">
         <f t="shared" si="14"/>

</xml_diff>